<commit_message>
Update Phone and Email
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Works\luzita\luzita-e-commers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC1FD6E6-021E-4409-B8EC-6CEB4EF7FBFC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0245DBF-9E16-4BC1-9B6B-6BA562EB4833}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Products" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="170">
   <si>
     <t>code</t>
   </si>
@@ -435,21 +435,12 @@
     <t>whatsapp</t>
   </si>
   <si>
-    <t>201001234567</t>
-  </si>
-  <si>
     <t>phone</t>
   </si>
   <si>
-    <t>01001234567</t>
-  </si>
-  <si>
     <t>email</t>
   </si>
   <si>
-    <t>info@luzita.store</t>
-  </si>
-  <si>
     <t>announcement</t>
   </si>
   <si>
@@ -538,6 +529,9 @@
   </si>
   <si>
     <t>images/categories/photo-1583743814966-8936f37f384c.jfif</t>
+  </si>
+  <si>
+    <t>samyalaa638@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -999,7 +993,7 @@
         <v>42</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
@@ -1040,7 +1034,7 @@
         <v>35</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
@@ -1081,7 +1075,7 @@
         <v>39</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
@@ -1122,7 +1116,7 @@
         <v>28</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
@@ -1163,7 +1157,7 @@
         <v>44</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
@@ -1204,7 +1198,7 @@
         <v>31</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
@@ -1245,7 +1239,7 @@
         <v>52</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
@@ -1286,7 +1280,7 @@
         <v>37</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
@@ -1327,7 +1321,7 @@
         <v>29</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
@@ -1368,7 +1362,7 @@
         <v>41</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
@@ -1409,7 +1403,7 @@
         <v>33</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
@@ -1450,7 +1444,7 @@
         <v>26</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
@@ -1491,7 +1485,7 @@
         <v>48</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
@@ -1532,7 +1526,7 @@
         <v>46</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
@@ -1573,7 +1567,7 @@
         <v>34</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
@@ -1614,7 +1608,7 @@
         <v>38</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.3">
@@ -1655,7 +1649,7 @@
         <v>27</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
@@ -1696,7 +1690,7 @@
         <v>32</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.3">
@@ -1737,7 +1731,7 @@
         <v>36</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.3">
@@ -1778,7 +1772,7 @@
         <v>43</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
@@ -1819,7 +1813,7 @@
         <v>31</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.3">
@@ -1860,7 +1854,7 @@
         <v>28</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
@@ -1901,7 +1895,7 @@
         <v>22</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.3">
@@ -1942,7 +1936,7 @@
         <v>25</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -2010,7 +2004,7 @@
         <v>125</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -2024,7 +2018,7 @@
         <v>126</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -2038,7 +2032,7 @@
         <v>127</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -2052,7 +2046,7 @@
         <v>128</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -2066,7 +2060,7 @@
         <v>129</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
   </sheetData>
@@ -2118,35 +2112,38 @@
       <c r="A4" t="s">
         <v>136</v>
       </c>
-      <c r="B4" t="s">
-        <v>137</v>
+      <c r="B4">
+        <v>1140993467</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>138</v>
-      </c>
-      <c r="B5" t="s">
-        <v>139</v>
+        <v>137</v>
+      </c>
+      <c r="B5">
+        <v>1140993467</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>140</v>
-      </c>
-      <c r="B6" t="s">
-        <v>141</v>
+        <v>138</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B7" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{EFE2586F-3CD0-42B5-AE95-2F70F70727EA}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>